<commit_message>
CI: actualizar bases, hojas y reportes
</commit_message>
<xml_diff>
--- a/_db/IMSA_DB.xlsx
+++ b/_db/IMSA_DB.xlsx
@@ -15733,7 +15733,7 @@
       <c r="E1" s="7"/>
       <c r="F1" s="1"/>
       <c r="G1" s="10">
-        <v>45945</v>
+        <v>45951</v>
       </c>
       <c r="H1" s="1"/>
       <c r="I1" s="1"/>
@@ -87464,8 +87464,8 @@
       <c r="G2320" s="9">
         <v>588000</v>
       </c>
-      <c r="H2320" s="6" t="s">
-        <v>45</v>
+      <c r="H2320" s="4" t="s">
+        <v>16</v>
       </c>
       <c r="J2320" s="9">
         <f t="shared" si="75"/>
@@ -87495,8 +87495,8 @@
       <c r="G2321" s="9">
         <v>448154</v>
       </c>
-      <c r="H2321" s="5" t="s">
-        <v>5080</v>
+      <c r="H2321" s="4" t="s">
+        <v>16</v>
       </c>
       <c r="J2321" s="9">
         <f t="shared" si="75"/>
@@ -87588,8 +87588,8 @@
       <c r="G2324" s="9">
         <v>1386000</v>
       </c>
-      <c r="H2324" s="5" t="s">
-        <v>5080</v>
+      <c r="H2324" s="4" t="s">
+        <v>16</v>
       </c>
       <c r="J2324" s="9">
         <f t="shared" si="75"/>
@@ -97140,7 +97140,7 @@
         <v>547</v>
       </c>
       <c r="E2633" s="9">
-        <f t="shared" ref="E2633:E2696" si="84">SUM(G2633/(1+(F2633/100)) /(1+(37/100)))</f>
+        <f t="shared" ref="E2633:E2658" si="84">SUM(G2633/(1+(F2633/100)) /(1+(37/100)))</f>
         <v>11333.775713337756</v>
       </c>
       <c r="F2633" s="3">
@@ -97153,7 +97153,7 @@
         <v>16</v>
       </c>
       <c r="J2633" s="9">
-        <f t="shared" ref="J2633:J2696" si="85">SUM(E2633* I2633)</f>
+        <f t="shared" ref="J2633:J2658" si="85">SUM(E2633* I2633)</f>
         <v>0</v>
       </c>
     </row>

</xml_diff>